<commit_message>
data preparation process committed
</commit_message>
<xml_diff>
--- a/Assets/Info_graphs/benchmark/required budget planning for APAM - 2025.12.10.xlsx
+++ b/Assets/Info_graphs/benchmark/required budget planning for APAM - 2025.12.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\01. IE (Industrial Engineering)\00. Univesity\Masters\05. Master's thesis\PPO-project-portfolio-budgeting-AI-agent\assets\Info_graphs\benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4BDB002-15DF-43C4-AD50-6911917DAB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626BA2E8-9F96-445D-A61B-D351F28CD0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC314A85-E3D9-49AD-A2B3-2D5D99045332}"/>
   </bookViews>
@@ -189,21 +189,63 @@
     <t>NO less than previous earned value on dedicated budget with 10% added safty</t>
   </si>
   <si>
-    <t>Prove that considering drawbacks and benifits of both sides and use weights for them to prove the agent is as good as the benchmark, which is knowing the future. 
+    <r>
+      <t xml:space="preserve">Prove that considering drawbacks and benifits of both sides and use weights for them to prove the agent is as good as the benchmark, which is knowing the future. 
 It's almost as good as the future. 
 * implementing convex optimization on allocation decisions over the portfolio timespan. knowing the future values and solving for optimal solution gives the ultimate benchmark to evaluate the agent's policy.
 * for evaluating the agent's policy we have to consider all the positive concervativeness of not knowing the future and increase the weghts of it's parameter in scoring it relative to the optimal solution.
-* the agent must establish obvious patterns of learning and then at the last 100 episodes we must evaluate it's response with the benchmark for those episodes and report the conclusion as a mean of the final states.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>* the agent must establish obvious patterns of learning and then at the last 100 episodes we must evaluate it's response with the benchmark for those episodes and report the conclusion as a mean of the final states.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
 ----
-Use the data from the previous year of S&amp;P500 for one implementation of uncertainty for payments as the market value is the best indicator of the major status of a company. also it's a relatively good data set.
-____</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Use the data from the previous year of S&amp;P500 for one implementation of uncertainty for payments as the market value is the best indicator of the major status of a company. also it's a relatively good data set.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>____</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,6 +291,27 @@
       <color rgb="FFFFC000"/>
       <name val="Cascadia Code SemiBold"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF00B050"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -436,7 +499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -525,10 +588,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1066,15 +1126,15 @@
       </c>
       <c r="K12" s="1">
         <f t="shared" ref="K12:K23" ca="1" si="0">(RANDBETWEEN(80,100)/100)</f>
-        <v>0.93</v>
+        <v>0.82</v>
       </c>
       <c r="L12" s="1">
         <f ca="1">K12*H12</f>
-        <v>4.4285714285714282E-2</v>
+        <v>3.9047619047619046E-2</v>
       </c>
       <c r="M12" s="2">
         <f ca="1">M11+L12</f>
-        <v>4.4285714285714282E-2</v>
+        <v>3.9047619047619046E-2</v>
       </c>
       <c r="O12" s="1">
         <f>I12-D12</f>
@@ -1082,19 +1142,19 @@
       </c>
       <c r="P12" s="1">
         <f ca="1">C12-L12</f>
-        <v>3.333333333333334E-3</v>
+        <v>8.5714285714285701E-3</v>
       </c>
       <c r="Q12" s="2">
         <f ca="1">D12-M12</f>
-        <v>3.333333333333334E-3</v>
+        <v>8.5714285714285701E-3</v>
       </c>
       <c r="S12" s="27">
         <f ca="1">M12/D12</f>
-        <v>0.92999999999999994</v>
+        <v>0.82000000000000006</v>
       </c>
       <c r="T12" s="26">
         <f ca="1">M12/I12</f>
-        <v>0.92999999999999994</v>
+        <v>0.82000000000000006</v>
       </c>
       <c r="U12" s="1"/>
     </row>
@@ -1111,51 +1171,51 @@
       </c>
       <c r="E13" s="2">
         <f ca="1">D13-M12</f>
-        <v>5.095238095238095E-2</v>
+        <v>5.6190476190476187E-2</v>
       </c>
       <c r="G13" s="1">
         <f ca="1">MIN($K$12:K13)-0.1</f>
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="H13" s="13">
         <f ca="1">E13/G13</f>
-        <v>6.8854568854568851E-2</v>
+        <v>7.8042328042328038E-2</v>
       </c>
       <c r="I13" s="2">
         <f ca="1">I12+H13</f>
-        <v>0.11647361647361647</v>
+        <v>0.12566137566137564</v>
       </c>
       <c r="K13" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="L13" s="1">
         <f t="shared" ref="L13" ca="1" si="1">K13*H13</f>
-        <v>5.783783783783783E-2</v>
+        <v>7.7261904761904754E-2</v>
       </c>
       <c r="M13" s="2">
         <f ca="1">M12+L13</f>
-        <v>0.10212355212355212</v>
+        <v>0.11630952380952381</v>
       </c>
       <c r="O13" s="1">
         <f ca="1">I13-D13</f>
-        <v>2.1235521235521235E-2</v>
+        <v>3.0423280423280408E-2</v>
       </c>
       <c r="P13" s="1">
         <f ca="1">C13-L13</f>
-        <v>-1.0218790218790214E-2</v>
+        <v>-2.9642857142857137E-2</v>
       </c>
       <c r="Q13" s="2">
         <f ca="1">D13-M13</f>
-        <v>-6.8854568854568865E-3</v>
+        <v>-2.1071428571428574E-2</v>
       </c>
       <c r="S13" s="27">
         <f ca="1">M13/D13</f>
-        <v>1.0722972972972973</v>
+        <v>1.2212499999999999</v>
       </c>
       <c r="T13" s="26">
         <f ca="1">M13/I13</f>
-        <v>0.8767955801104973</v>
+        <v>0.92557894736842117</v>
       </c>
       <c r="U13" s="1"/>
     </row>
@@ -1172,51 +1232,51 @@
       </c>
       <c r="E14" s="2">
         <f t="shared" ref="E14:E22" ca="1" si="3">D14-M13</f>
-        <v>4.073359073359073E-2</v>
+        <v>2.6547619047619042E-2</v>
       </c>
       <c r="G14" s="1">
         <f ca="1">MIN($K$12:K14)-0.1</f>
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="H14" s="13">
         <f t="shared" ref="H14:H22" ca="1" si="4">E14/G14</f>
-        <v>5.5045392883230716E-2</v>
+        <v>3.6871693121693118E-2</v>
       </c>
       <c r="I14" s="2">
         <f t="shared" ref="I14:I23" ca="1" si="5">I13+H14</f>
-        <v>0.17151900935684719</v>
+        <v>0.16253306878306875</v>
       </c>
       <c r="K14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="L14" s="1">
         <f t="shared" ref="L14:L22" ca="1" si="6">K14*H14</f>
-        <v>4.8990399666075338E-2</v>
+        <v>3.2078373015873012E-2</v>
       </c>
       <c r="M14" s="2">
         <f t="shared" ref="M14:M22" ca="1" si="7">M13+L14</f>
-        <v>0.15111395178962744</v>
+        <v>0.14838789682539683</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" ref="O14:O22" ca="1" si="8">I14-D14</f>
-        <v>2.8661866499704342E-2</v>
+        <v>1.9675925925925902E-2</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" ref="P14:P22" ca="1" si="9">C14-L14</f>
-        <v>-1.3713520470277213E-3</v>
+        <v>1.5540674603174605E-2</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" ref="Q14:Q22" ca="1" si="10">D14-M14</f>
-        <v>-8.2568089324845939E-3</v>
+        <v>-5.5307539682539764E-3</v>
       </c>
       <c r="S14" s="27">
         <f t="shared" ref="S14:S22" ca="1" si="11">M14/D14</f>
-        <v>1.0577976625273922</v>
+        <v>1.0387152777777779</v>
       </c>
       <c r="T14" s="26">
         <f t="shared" ref="T14:T22" ca="1" si="12">M14/I14</f>
-        <v>0.88103325897383888</v>
+        <v>0.9129704984740592</v>
       </c>
       <c r="U14" s="1"/>
     </row>
@@ -1233,51 +1293,51 @@
       </c>
       <c r="E15" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>8.6981286305610639E-2</v>
+        <v>8.9707341269841256E-2</v>
       </c>
       <c r="G15" s="1">
         <f ca="1">MIN($K$12:K15)-0.1</f>
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="H15" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>0.11754227879136572</v>
+        <v>0.12459352954144619</v>
       </c>
       <c r="I15" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.28906128814821291</v>
+        <v>0.28712659832451493</v>
       </c>
       <c r="K15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="L15" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>9.87355141847472E-2</v>
+        <v>0.10964230599647265</v>
       </c>
       <c r="M15" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.24984946597437463</v>
+        <v>0.2580302028218695</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>5.0966050052974832E-2</v>
+        <v>4.9031360229276844E-2</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-3.4974189466519673E-3</v>
+        <v>-1.4404210758377417E-2</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-1.1754227879136547E-2</v>
+        <v>-1.9934964726631421E-2</v>
       </c>
       <c r="S15" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0493677570923734</v>
+        <v>1.0837268518518519</v>
       </c>
       <c r="T15" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.86434772215595723</v>
+        <v>0.89866353144420208</v>
       </c>
       <c r="U15" s="1"/>
     </row>
@@ -1294,51 +1354,51 @@
       </c>
       <c r="E16" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>8.3483867358958685E-2</v>
+        <v>7.5303130511463812E-2</v>
       </c>
       <c r="G16" s="1">
         <f ca="1">MIN($K$12:K16)-0.1</f>
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="H16" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>0.11281603697156579</v>
+        <v>0.10458768126592197</v>
       </c>
       <c r="I16" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.40187732511977869</v>
+        <v>0.39171427959043692</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>9.9278112534977897E-2</v>
+        <v>9.9358297202625859E-2</v>
       </c>
       <c r="M16" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.3491275785093525</v>
+        <v>0.35738850002449535</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>6.854399178644538E-2</v>
+        <v>5.8380946257103605E-2</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-4.0400172968826642E-3</v>
+        <v>-4.1202019645306259E-3</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-1.5794245176019184E-2</v>
+        <v>-2.4055166691162033E-2</v>
       </c>
       <c r="S16" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0473827355280576</v>
+        <v>1.0721655000734862</v>
       </c>
       <c r="T16" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.86874166987474533</v>
+        <v>0.91237036443544661</v>
       </c>
       <c r="U16" s="1"/>
     </row>
@@ -1355,51 +1415,51 @@
       </c>
       <c r="E17" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>0.12706289768112367</v>
+        <v>0.11880197616598082</v>
       </c>
       <c r="G17" s="1">
         <f ca="1">MIN($K$12:K17)-0.1</f>
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="H17" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>0.17405876394674474</v>
+        <v>0.16500274467497336</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.57593608906652349</v>
+        <v>0.55671702426541025</v>
       </c>
       <c r="K17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="L17" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0.14446877407579814</v>
+        <v>0.1419023604204771</v>
       </c>
       <c r="M17" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.49359635258515067</v>
+        <v>0.49929086044497245</v>
       </c>
       <c r="O17" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>9.9745612876047329E-2</v>
+        <v>8.052654807493409E-2</v>
       </c>
       <c r="P17" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.6116312186552906E-3</v>
+        <v>9.5478243666574647E-4</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-1.7405876394674502E-2</v>
+        <v>-2.3100384254496287E-2</v>
       </c>
       <c r="S17" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0365523404288164</v>
+        <v>1.0485108069344422</v>
       </c>
       <c r="T17" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.85703320551620754</v>
+        <v>0.8968485580332094</v>
       </c>
       <c r="U17" s="1"/>
     </row>
@@ -1416,7 +1476,7 @@
       </c>
       <c r="E18" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>0.1254512664624684</v>
+        <v>0.11975675860264662</v>
       </c>
       <c r="G18" s="1">
         <f ca="1">MIN($K$12:K18)-0.1</f>
@@ -1424,43 +1484,43 @@
       </c>
       <c r="H18" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>0.17423787008676167</v>
+        <v>0.16632883139256474</v>
       </c>
       <c r="I18" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.75017395915328522</v>
+        <v>0.72304585565797497</v>
       </c>
       <c r="K18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82</v>
+        <v>0.94</v>
       </c>
       <c r="L18" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0.14287505347114457</v>
+        <v>0.15634910150901085</v>
       </c>
       <c r="M18" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.63647140605629526</v>
+        <v>0.65563996195398333</v>
       </c>
       <c r="O18" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>0.13112634010566615</v>
+        <v>0.1039982366103559</v>
       </c>
       <c r="P18" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.7910614001720448E-5</v>
+        <v>-1.3491958651868002E-2</v>
       </c>
       <c r="Q18" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-1.7423787008676195E-2</v>
+        <v>-3.6592342906364261E-2</v>
       </c>
       <c r="S18" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.028146117475554</v>
+        <v>1.0591107077718191</v>
       </c>
       <c r="T18" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.84843175144959038</v>
+        <v>0.90677507771253041</v>
       </c>
       <c r="U18" s="1"/>
     </row>
@@ -1477,7 +1537,7 @@
       </c>
       <c r="E19" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>0.1254333558484666</v>
+        <v>0.10626479995077853</v>
       </c>
       <c r="G19" s="1">
         <f ca="1">MIN($K$12:K19)-0.1</f>
@@ -1485,43 +1545,43 @@
       </c>
       <c r="H19" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>0.1742129942339814</v>
+        <v>0.14758999993163685</v>
       </c>
       <c r="I19" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.92438695338726662</v>
+        <v>0.87063585558961187</v>
       </c>
       <c r="K19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="L19" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0.16898660440696195</v>
+        <v>0.14758999993163685</v>
       </c>
       <c r="M19" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.80545801046325716</v>
+        <v>0.80322996188562024</v>
       </c>
       <c r="O19" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>0.16248219148250476</v>
+        <v>0.10873109368485001</v>
       </c>
       <c r="P19" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-2.61294615498191E-2</v>
+        <v>-4.7328570744940013E-3</v>
       </c>
       <c r="Q19" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-4.3553248558495294E-2</v>
+        <v>-4.1325199980858374E-2</v>
       </c>
       <c r="S19" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.057163638733025</v>
+        <v>1.0542393249748767</v>
       </c>
       <c r="T19" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.8713429019219564</v>
+        <v>0.92257854616113522</v>
       </c>
       <c r="U19" s="1"/>
     </row>
@@ -1538,7 +1598,7 @@
       </c>
       <c r="E20" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>5.1684846679599938E-2</v>
+        <v>5.3912895257236859E-2</v>
       </c>
       <c r="G20" s="1">
         <f ca="1">MIN($K$12:K20)-0.1</f>
@@ -1546,43 +1606,43 @@
       </c>
       <c r="H20" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>7.1784509277222144E-2</v>
+        <v>7.4879021190606757E-2</v>
       </c>
       <c r="I20" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>0.99617146266448875</v>
+        <v>0.94551487678021862</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.99</v>
+        <v>0.94</v>
       </c>
       <c r="L20" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>7.1066664184449929E-2</v>
+        <v>7.0386279919170347E-2</v>
       </c>
       <c r="M20" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.87652467464770711</v>
+        <v>0.87361624180479058</v>
       </c>
       <c r="O20" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>0.13902860552163165</v>
+        <v>8.8372019637361521E-2</v>
       </c>
       <c r="P20" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>2.4171431053645304E-2</v>
+        <v>2.4851815318924886E-2</v>
       </c>
       <c r="Q20" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-1.9381817504850019E-2</v>
+        <v>-1.6473384661933488E-2</v>
       </c>
       <c r="S20" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0226121204223251</v>
+        <v>1.0192189487722558</v>
       </c>
       <c r="T20" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.87989337930163258</v>
+        <v>0.92395821922943622</v>
       </c>
       <c r="U20" s="1"/>
     </row>
@@ -1599,51 +1659,51 @@
       </c>
       <c r="E21" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>2.8237230114197542E-2</v>
+        <v>3.1145662957114073E-2</v>
       </c>
       <c r="G21" s="1">
         <f ca="1">MIN($K$12:K21)-0.1</f>
-        <v>0.72</v>
+        <v>0.71000000000000008</v>
       </c>
       <c r="H21" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>3.9218375158607696E-2</v>
+        <v>4.3867130925512775E-2</v>
       </c>
       <c r="I21" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>1.0353898378230963</v>
+        <v>0.98938200770573137</v>
       </c>
       <c r="K21" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.88</v>
+        <v>0.81</v>
       </c>
       <c r="L21" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>3.451217013957477E-2</v>
+        <v>3.5532376049665353E-2</v>
       </c>
       <c r="M21" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.91103684478728186</v>
+        <v>0.90914861785445589</v>
       </c>
       <c r="O21" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>0.13062793306119169</v>
+        <v>8.4620102943826714E-2</v>
       </c>
       <c r="P21" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>1.3106877479472846E-2</v>
+        <v>1.2086671569382264E-2</v>
       </c>
       <c r="Q21" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-6.274940025377207E-3</v>
+        <v>-4.386713092551231E-3</v>
       </c>
       <c r="S21" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0069354600280485</v>
+        <v>1.0048484723654514</v>
       </c>
       <c r="T21" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.87989741786797304</v>
+        <v>0.91890554990248108</v>
       </c>
       <c r="U21" s="1"/>
     </row>
@@ -1660,51 +1720,51 @@
       </c>
       <c r="E22" s="2">
         <f t="shared" ca="1" si="3"/>
-        <v>4.1344107593670465E-2</v>
+        <v>4.3232334526496441E-2</v>
       </c>
       <c r="G22" s="1">
         <f ca="1">MIN($K$12:K22)-0.1</f>
-        <v>0.72</v>
+        <v>0.71000000000000008</v>
       </c>
       <c r="H22" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>5.742237165787565E-2</v>
+        <v>6.0890612009149914E-2</v>
       </c>
       <c r="I22" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>1.092812209480972</v>
+        <v>1.0502726197148813</v>
       </c>
       <c r="K22" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="L22" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>4.7660568476036787E-2</v>
+        <v>5.2365926327868927E-2</v>
       </c>
       <c r="M22" s="2">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9586974132633187</v>
+        <v>0.96151454418232485</v>
       </c>
       <c r="O22" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>0.14043125710001969</v>
+        <v>9.7891667333928956E-2</v>
       </c>
       <c r="P22" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-4.1520856989170352E-5</v>
+        <v>-4.7468787088213102E-3</v>
       </c>
       <c r="Q22" s="2">
         <f t="shared" ca="1" si="10"/>
-        <v>-6.3164608823663704E-3</v>
+        <v>-9.1335918013725204E-3</v>
       </c>
       <c r="S22" s="27">
         <f t="shared" ca="1" si="11"/>
-        <v>1.0066322839264847</v>
+        <v>1.0095902713914411</v>
       </c>
       <c r="T22" s="26">
         <f t="shared" ca="1" si="12"/>
-        <v>0.87727553274560255</v>
+        <v>0.91549044137068747</v>
       </c>
       <c r="U22" s="1"/>
     </row>
@@ -1721,51 +1781,51 @@
       </c>
       <c r="E23" s="2">
         <f t="shared" ref="E23" ca="1" si="14">D23-M22</f>
-        <v>4.1302586736681302E-2</v>
+        <v>3.8485455817675152E-2</v>
       </c>
       <c r="G23" s="1">
         <f ca="1">MIN($K$12:K23)-0.1</f>
-        <v>0.72</v>
+        <v>0.71000000000000008</v>
       </c>
       <c r="H23" s="13">
         <f t="shared" ref="H23" ca="1" si="15">E23/G23</f>
-        <v>5.7364703800946257E-2</v>
+        <v>5.4204867348838233E-2</v>
       </c>
       <c r="I23" s="2">
         <f t="shared" ca="1" si="5"/>
-        <v>1.1501769132819182</v>
+        <v>1.1044774870637195</v>
       </c>
       <c r="K23" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.92</v>
+        <v>0.89</v>
       </c>
       <c r="L23" s="1">
         <f t="shared" ref="L23" ca="1" si="16">K23*H23</f>
-        <v>5.2775527496870561E-2</v>
+        <v>4.8242331940466031E-2</v>
       </c>
       <c r="M23" s="2">
         <f t="shared" ref="M23" ca="1" si="17">M22+L23</f>
-        <v>1.0114729407601892</v>
+        <v>1.0097568761227909</v>
       </c>
       <c r="O23" s="1">
         <f t="shared" ref="O23" ca="1" si="18">I23-D23</f>
-        <v>0.15017691328191818</v>
+        <v>0.10447748706371951</v>
       </c>
       <c r="P23" s="1">
         <f t="shared" ref="P23" ca="1" si="19">C23-L23</f>
-        <v>-5.1564798778229448E-3</v>
+        <v>-6.2328432141841444E-4</v>
       </c>
       <c r="Q23" s="2">
         <f t="shared" ref="Q23" ca="1" si="20">D23-M23</f>
-        <v>-1.1472940760189232E-2</v>
+        <v>-9.7568761227908585E-3</v>
       </c>
       <c r="S23" s="27">
         <f t="shared" ref="S23" ca="1" si="21">M23/D23</f>
-        <v>1.0114729407601892</v>
+        <v>1.0097568761227909</v>
       </c>
       <c r="T23" s="26">
         <f t="shared" ref="T23" ca="1" si="22">M23/I23</f>
-        <v>0.87940640181522112</v>
+        <v>0.91423943715435463</v>
       </c>
       <c r="U23" s="1"/>
     </row>
@@ -1784,7 +1844,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16">
         <f ca="1">SUM(H11:H23)</f>
-        <v>1.1501769132819182</v>
+        <v>1.1044774870637195</v>
       </c>
       <c r="I24" s="17" t="b">
         <f ca="1">I23=H24</f>
@@ -1794,7 +1854,7 @@
       <c r="K24" s="16"/>
       <c r="L24" s="28">
         <f ca="1">SUM(L11:L23)</f>
-        <v>1.0114729407601892</v>
+        <v>1.0097568761227909</v>
       </c>
       <c r="M24" s="17" t="b">
         <f ca="1">M23=L24</f>
@@ -2517,383 +2577,383 @@
       <c r="C66" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D66" s="31"/>
-      <c r="E66" s="31"/>
-      <c r="F66" s="31"/>
-      <c r="G66" s="31"/>
-      <c r="H66" s="31"/>
-      <c r="I66" s="31"/>
-      <c r="J66" s="31"/>
-      <c r="K66" s="31"/>
-      <c r="L66" s="31"/>
-      <c r="M66" s="31"/>
-      <c r="N66" s="31"/>
-      <c r="O66" s="31"/>
-      <c r="P66" s="31"/>
-      <c r="Q66" s="31"/>
-      <c r="R66" s="31"/>
-      <c r="S66" s="31"/>
+      <c r="D66" s="30"/>
+      <c r="E66" s="30"/>
+      <c r="F66" s="30"/>
+      <c r="G66" s="30"/>
+      <c r="H66" s="30"/>
+      <c r="I66" s="30"/>
+      <c r="J66" s="30"/>
+      <c r="K66" s="30"/>
+      <c r="L66" s="30"/>
+      <c r="M66" s="30"/>
+      <c r="N66" s="30"/>
+      <c r="O66" s="30"/>
+      <c r="P66" s="30"/>
+      <c r="Q66" s="30"/>
+      <c r="R66" s="30"/>
+      <c r="S66" s="30"/>
     </row>
     <row r="67" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="31"/>
-      <c r="H67" s="31"/>
-      <c r="I67" s="31"/>
-      <c r="J67" s="31"/>
-      <c r="K67" s="31"/>
-      <c r="L67" s="31"/>
-      <c r="M67" s="31"/>
-      <c r="N67" s="31"/>
-      <c r="O67" s="31"/>
-      <c r="P67" s="31"/>
-      <c r="Q67" s="31"/>
-      <c r="R67" s="31"/>
-      <c r="S67" s="31"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="30"/>
+      <c r="E67" s="30"/>
+      <c r="F67" s="30"/>
+      <c r="G67" s="30"/>
+      <c r="H67" s="30"/>
+      <c r="I67" s="30"/>
+      <c r="J67" s="30"/>
+      <c r="K67" s="30"/>
+      <c r="L67" s="30"/>
+      <c r="M67" s="30"/>
+      <c r="N67" s="30"/>
+      <c r="O67" s="30"/>
+      <c r="P67" s="30"/>
+      <c r="Q67" s="30"/>
+      <c r="R67" s="30"/>
+      <c r="S67" s="30"/>
     </row>
     <row r="68" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C68" s="31"/>
-      <c r="D68" s="31"/>
-      <c r="E68" s="31"/>
-      <c r="F68" s="31"/>
-      <c r="G68" s="31"/>
-      <c r="H68" s="31"/>
-      <c r="I68" s="31"/>
-      <c r="J68" s="31"/>
-      <c r="K68" s="31"/>
-      <c r="L68" s="31"/>
-      <c r="M68" s="31"/>
-      <c r="N68" s="31"/>
-      <c r="O68" s="31"/>
-      <c r="P68" s="31"/>
-      <c r="Q68" s="31"/>
-      <c r="R68" s="31"/>
-      <c r="S68" s="31"/>
+      <c r="C68" s="30"/>
+      <c r="D68" s="30"/>
+      <c r="E68" s="30"/>
+      <c r="F68" s="30"/>
+      <c r="G68" s="30"/>
+      <c r="H68" s="30"/>
+      <c r="I68" s="30"/>
+      <c r="J68" s="30"/>
+      <c r="K68" s="30"/>
+      <c r="L68" s="30"/>
+      <c r="M68" s="30"/>
+      <c r="N68" s="30"/>
+      <c r="O68" s="30"/>
+      <c r="P68" s="30"/>
+      <c r="Q68" s="30"/>
+      <c r="R68" s="30"/>
+      <c r="S68" s="30"/>
     </row>
     <row r="69" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C69" s="31"/>
-      <c r="D69" s="31"/>
-      <c r="E69" s="31"/>
-      <c r="F69" s="31"/>
-      <c r="G69" s="31"/>
-      <c r="H69" s="31"/>
-      <c r="I69" s="31"/>
-      <c r="J69" s="31"/>
-      <c r="K69" s="31"/>
-      <c r="L69" s="31"/>
-      <c r="M69" s="31"/>
-      <c r="N69" s="31"/>
-      <c r="O69" s="31"/>
-      <c r="P69" s="31"/>
-      <c r="Q69" s="31"/>
-      <c r="R69" s="31"/>
-      <c r="S69" s="31"/>
+      <c r="C69" s="30"/>
+      <c r="D69" s="30"/>
+      <c r="E69" s="30"/>
+      <c r="F69" s="30"/>
+      <c r="G69" s="30"/>
+      <c r="H69" s="30"/>
+      <c r="I69" s="30"/>
+      <c r="J69" s="30"/>
+      <c r="K69" s="30"/>
+      <c r="L69" s="30"/>
+      <c r="M69" s="30"/>
+      <c r="N69" s="30"/>
+      <c r="O69" s="30"/>
+      <c r="P69" s="30"/>
+      <c r="Q69" s="30"/>
+      <c r="R69" s="30"/>
+      <c r="S69" s="30"/>
     </row>
     <row r="70" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C70" s="31"/>
-      <c r="D70" s="31"/>
-      <c r="E70" s="31"/>
-      <c r="F70" s="31"/>
-      <c r="G70" s="31"/>
-      <c r="H70" s="31"/>
-      <c r="I70" s="31"/>
-      <c r="J70" s="31"/>
-      <c r="K70" s="31"/>
-      <c r="L70" s="31"/>
-      <c r="M70" s="31"/>
-      <c r="N70" s="31"/>
-      <c r="O70" s="31"/>
-      <c r="P70" s="31"/>
-      <c r="Q70" s="31"/>
-      <c r="R70" s="31"/>
-      <c r="S70" s="31"/>
+      <c r="C70" s="30"/>
+      <c r="D70" s="30"/>
+      <c r="E70" s="30"/>
+      <c r="F70" s="30"/>
+      <c r="G70" s="30"/>
+      <c r="H70" s="30"/>
+      <c r="I70" s="30"/>
+      <c r="J70" s="30"/>
+      <c r="K70" s="30"/>
+      <c r="L70" s="30"/>
+      <c r="M70" s="30"/>
+      <c r="N70" s="30"/>
+      <c r="O70" s="30"/>
+      <c r="P70" s="30"/>
+      <c r="Q70" s="30"/>
+      <c r="R70" s="30"/>
+      <c r="S70" s="30"/>
     </row>
     <row r="71" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C71" s="31"/>
-      <c r="D71" s="31"/>
-      <c r="E71" s="31"/>
-      <c r="F71" s="31"/>
-      <c r="G71" s="31"/>
-      <c r="H71" s="31"/>
-      <c r="I71" s="31"/>
-      <c r="J71" s="31"/>
-      <c r="K71" s="31"/>
-      <c r="L71" s="31"/>
-      <c r="M71" s="31"/>
-      <c r="N71" s="31"/>
-      <c r="O71" s="31"/>
-      <c r="P71" s="31"/>
-      <c r="Q71" s="31"/>
-      <c r="R71" s="31"/>
-      <c r="S71" s="31"/>
+      <c r="C71" s="30"/>
+      <c r="D71" s="30"/>
+      <c r="E71" s="30"/>
+      <c r="F71" s="30"/>
+      <c r="G71" s="30"/>
+      <c r="H71" s="30"/>
+      <c r="I71" s="30"/>
+      <c r="J71" s="30"/>
+      <c r="K71" s="30"/>
+      <c r="L71" s="30"/>
+      <c r="M71" s="30"/>
+      <c r="N71" s="30"/>
+      <c r="O71" s="30"/>
+      <c r="P71" s="30"/>
+      <c r="Q71" s="30"/>
+      <c r="R71" s="30"/>
+      <c r="S71" s="30"/>
     </row>
     <row r="72" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C72" s="31"/>
-      <c r="D72" s="31"/>
-      <c r="E72" s="31"/>
-      <c r="F72" s="31"/>
-      <c r="G72" s="31"/>
-      <c r="H72" s="31"/>
-      <c r="I72" s="31"/>
-      <c r="J72" s="31"/>
-      <c r="K72" s="31"/>
-      <c r="L72" s="31"/>
-      <c r="M72" s="31"/>
-      <c r="N72" s="31"/>
-      <c r="O72" s="31"/>
-      <c r="P72" s="31"/>
-      <c r="Q72" s="31"/>
-      <c r="R72" s="31"/>
-      <c r="S72" s="31"/>
+      <c r="C72" s="30"/>
+      <c r="D72" s="30"/>
+      <c r="E72" s="30"/>
+      <c r="F72" s="30"/>
+      <c r="G72" s="30"/>
+      <c r="H72" s="30"/>
+      <c r="I72" s="30"/>
+      <c r="J72" s="30"/>
+      <c r="K72" s="30"/>
+      <c r="L72" s="30"/>
+      <c r="M72" s="30"/>
+      <c r="N72" s="30"/>
+      <c r="O72" s="30"/>
+      <c r="P72" s="30"/>
+      <c r="Q72" s="30"/>
+      <c r="R72" s="30"/>
+      <c r="S72" s="30"/>
     </row>
     <row r="73" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C73" s="31"/>
-      <c r="D73" s="31"/>
-      <c r="E73" s="31"/>
-      <c r="F73" s="31"/>
-      <c r="G73" s="31"/>
-      <c r="H73" s="31"/>
-      <c r="I73" s="31"/>
-      <c r="J73" s="31"/>
-      <c r="K73" s="31"/>
-      <c r="L73" s="31"/>
-      <c r="M73" s="31"/>
-      <c r="N73" s="31"/>
-      <c r="O73" s="31"/>
-      <c r="P73" s="31"/>
-      <c r="Q73" s="31"/>
-      <c r="R73" s="31"/>
-      <c r="S73" s="31"/>
+      <c r="C73" s="30"/>
+      <c r="D73" s="30"/>
+      <c r="E73" s="30"/>
+      <c r="F73" s="30"/>
+      <c r="G73" s="30"/>
+      <c r="H73" s="30"/>
+      <c r="I73" s="30"/>
+      <c r="J73" s="30"/>
+      <c r="K73" s="30"/>
+      <c r="L73" s="30"/>
+      <c r="M73" s="30"/>
+      <c r="N73" s="30"/>
+      <c r="O73" s="30"/>
+      <c r="P73" s="30"/>
+      <c r="Q73" s="30"/>
+      <c r="R73" s="30"/>
+      <c r="S73" s="30"/>
     </row>
     <row r="74" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C74" s="31"/>
-      <c r="D74" s="31"/>
-      <c r="E74" s="31"/>
-      <c r="F74" s="31"/>
-      <c r="G74" s="31"/>
-      <c r="H74" s="31"/>
-      <c r="I74" s="31"/>
-      <c r="J74" s="31"/>
-      <c r="K74" s="31"/>
-      <c r="L74" s="31"/>
-      <c r="M74" s="31"/>
-      <c r="N74" s="31"/>
-      <c r="O74" s="31"/>
-      <c r="P74" s="31"/>
-      <c r="Q74" s="31"/>
-      <c r="R74" s="31"/>
-      <c r="S74" s="31"/>
+      <c r="C74" s="30"/>
+      <c r="D74" s="30"/>
+      <c r="E74" s="30"/>
+      <c r="F74" s="30"/>
+      <c r="G74" s="30"/>
+      <c r="H74" s="30"/>
+      <c r="I74" s="30"/>
+      <c r="J74" s="30"/>
+      <c r="K74" s="30"/>
+      <c r="L74" s="30"/>
+      <c r="M74" s="30"/>
+      <c r="N74" s="30"/>
+      <c r="O74" s="30"/>
+      <c r="P74" s="30"/>
+      <c r="Q74" s="30"/>
+      <c r="R74" s="30"/>
+      <c r="S74" s="30"/>
     </row>
     <row r="75" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C75" s="31"/>
-      <c r="D75" s="31"/>
-      <c r="E75" s="31"/>
-      <c r="F75" s="31"/>
-      <c r="G75" s="31"/>
-      <c r="H75" s="31"/>
-      <c r="I75" s="31"/>
-      <c r="J75" s="31"/>
-      <c r="K75" s="31"/>
-      <c r="L75" s="31"/>
-      <c r="M75" s="31"/>
-      <c r="N75" s="31"/>
-      <c r="O75" s="31"/>
-      <c r="P75" s="31"/>
-      <c r="Q75" s="31"/>
-      <c r="R75" s="31"/>
-      <c r="S75" s="31"/>
+      <c r="C75" s="30"/>
+      <c r="D75" s="30"/>
+      <c r="E75" s="30"/>
+      <c r="F75" s="30"/>
+      <c r="G75" s="30"/>
+      <c r="H75" s="30"/>
+      <c r="I75" s="30"/>
+      <c r="J75" s="30"/>
+      <c r="K75" s="30"/>
+      <c r="L75" s="30"/>
+      <c r="M75" s="30"/>
+      <c r="N75" s="30"/>
+      <c r="O75" s="30"/>
+      <c r="P75" s="30"/>
+      <c r="Q75" s="30"/>
+      <c r="R75" s="30"/>
+      <c r="S75" s="30"/>
     </row>
     <row r="76" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C76" s="31"/>
-      <c r="D76" s="31"/>
-      <c r="E76" s="31"/>
-      <c r="F76" s="31"/>
-      <c r="G76" s="31"/>
-      <c r="H76" s="31"/>
-      <c r="I76" s="31"/>
-      <c r="J76" s="31"/>
-      <c r="K76" s="31"/>
-      <c r="L76" s="31"/>
-      <c r="M76" s="31"/>
-      <c r="N76" s="31"/>
-      <c r="O76" s="31"/>
-      <c r="P76" s="31"/>
-      <c r="Q76" s="31"/>
-      <c r="R76" s="31"/>
-      <c r="S76" s="31"/>
+      <c r="C76" s="30"/>
+      <c r="D76" s="30"/>
+      <c r="E76" s="30"/>
+      <c r="F76" s="30"/>
+      <c r="G76" s="30"/>
+      <c r="H76" s="30"/>
+      <c r="I76" s="30"/>
+      <c r="J76" s="30"/>
+      <c r="K76" s="30"/>
+      <c r="L76" s="30"/>
+      <c r="M76" s="30"/>
+      <c r="N76" s="30"/>
+      <c r="O76" s="30"/>
+      <c r="P76" s="30"/>
+      <c r="Q76" s="30"/>
+      <c r="R76" s="30"/>
+      <c r="S76" s="30"/>
     </row>
     <row r="77" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C77" s="31"/>
-      <c r="D77" s="31"/>
-      <c r="E77" s="31"/>
-      <c r="F77" s="31"/>
-      <c r="G77" s="31"/>
-      <c r="H77" s="31"/>
-      <c r="I77" s="31"/>
-      <c r="J77" s="31"/>
-      <c r="K77" s="31"/>
-      <c r="L77" s="31"/>
-      <c r="M77" s="31"/>
-      <c r="N77" s="31"/>
-      <c r="O77" s="31"/>
-      <c r="P77" s="31"/>
-      <c r="Q77" s="31"/>
-      <c r="R77" s="31"/>
-      <c r="S77" s="31"/>
+      <c r="C77" s="30"/>
+      <c r="D77" s="30"/>
+      <c r="E77" s="30"/>
+      <c r="F77" s="30"/>
+      <c r="G77" s="30"/>
+      <c r="H77" s="30"/>
+      <c r="I77" s="30"/>
+      <c r="J77" s="30"/>
+      <c r="K77" s="30"/>
+      <c r="L77" s="30"/>
+      <c r="M77" s="30"/>
+      <c r="N77" s="30"/>
+      <c r="O77" s="30"/>
+      <c r="P77" s="30"/>
+      <c r="Q77" s="30"/>
+      <c r="R77" s="30"/>
+      <c r="S77" s="30"/>
     </row>
     <row r="78" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C78" s="31"/>
-      <c r="D78" s="31"/>
-      <c r="E78" s="31"/>
-      <c r="F78" s="31"/>
-      <c r="G78" s="31"/>
-      <c r="H78" s="31"/>
-      <c r="I78" s="31"/>
-      <c r="J78" s="31"/>
-      <c r="K78" s="31"/>
-      <c r="L78" s="31"/>
-      <c r="M78" s="31"/>
-      <c r="N78" s="31"/>
-      <c r="O78" s="31"/>
-      <c r="P78" s="31"/>
-      <c r="Q78" s="31"/>
-      <c r="R78" s="31"/>
-      <c r="S78" s="31"/>
+      <c r="C78" s="30"/>
+      <c r="D78" s="30"/>
+      <c r="E78" s="30"/>
+      <c r="F78" s="30"/>
+      <c r="G78" s="30"/>
+      <c r="H78" s="30"/>
+      <c r="I78" s="30"/>
+      <c r="J78" s="30"/>
+      <c r="K78" s="30"/>
+      <c r="L78" s="30"/>
+      <c r="M78" s="30"/>
+      <c r="N78" s="30"/>
+      <c r="O78" s="30"/>
+      <c r="P78" s="30"/>
+      <c r="Q78" s="30"/>
+      <c r="R78" s="30"/>
+      <c r="S78" s="30"/>
     </row>
     <row r="79" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C79" s="31"/>
-      <c r="D79" s="31"/>
-      <c r="E79" s="31"/>
-      <c r="F79" s="31"/>
-      <c r="G79" s="31"/>
-      <c r="H79" s="31"/>
-      <c r="I79" s="31"/>
-      <c r="J79" s="31"/>
-      <c r="K79" s="31"/>
-      <c r="L79" s="31"/>
-      <c r="M79" s="31"/>
-      <c r="N79" s="31"/>
-      <c r="O79" s="31"/>
-      <c r="P79" s="31"/>
-      <c r="Q79" s="31"/>
-      <c r="R79" s="31"/>
-      <c r="S79" s="31"/>
+      <c r="C79" s="30"/>
+      <c r="D79" s="30"/>
+      <c r="E79" s="30"/>
+      <c r="F79" s="30"/>
+      <c r="G79" s="30"/>
+      <c r="H79" s="30"/>
+      <c r="I79" s="30"/>
+      <c r="J79" s="30"/>
+      <c r="K79" s="30"/>
+      <c r="L79" s="30"/>
+      <c r="M79" s="30"/>
+      <c r="N79" s="30"/>
+      <c r="O79" s="30"/>
+      <c r="P79" s="30"/>
+      <c r="Q79" s="30"/>
+      <c r="R79" s="30"/>
+      <c r="S79" s="30"/>
     </row>
     <row r="80" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C80" s="31"/>
-      <c r="D80" s="31"/>
-      <c r="E80" s="31"/>
-      <c r="F80" s="31"/>
-      <c r="G80" s="31"/>
-      <c r="H80" s="31"/>
-      <c r="I80" s="31"/>
-      <c r="J80" s="31"/>
-      <c r="K80" s="31"/>
-      <c r="L80" s="31"/>
-      <c r="M80" s="31"/>
-      <c r="N80" s="31"/>
-      <c r="O80" s="31"/>
-      <c r="P80" s="31"/>
-      <c r="Q80" s="31"/>
-      <c r="R80" s="31"/>
-      <c r="S80" s="31"/>
+      <c r="C80" s="30"/>
+      <c r="D80" s="30"/>
+      <c r="E80" s="30"/>
+      <c r="F80" s="30"/>
+      <c r="G80" s="30"/>
+      <c r="H80" s="30"/>
+      <c r="I80" s="30"/>
+      <c r="J80" s="30"/>
+      <c r="K80" s="30"/>
+      <c r="L80" s="30"/>
+      <c r="M80" s="30"/>
+      <c r="N80" s="30"/>
+      <c r="O80" s="30"/>
+      <c r="P80" s="30"/>
+      <c r="Q80" s="30"/>
+      <c r="R80" s="30"/>
+      <c r="S80" s="30"/>
     </row>
     <row r="81" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C81" s="31"/>
-      <c r="D81" s="31"/>
-      <c r="E81" s="31"/>
-      <c r="F81" s="31"/>
-      <c r="G81" s="31"/>
-      <c r="H81" s="31"/>
-      <c r="I81" s="31"/>
-      <c r="J81" s="31"/>
-      <c r="K81" s="31"/>
-      <c r="L81" s="31"/>
-      <c r="M81" s="31"/>
-      <c r="N81" s="31"/>
-      <c r="O81" s="31"/>
-      <c r="P81" s="31"/>
-      <c r="Q81" s="31"/>
-      <c r="R81" s="31"/>
-      <c r="S81" s="31"/>
+      <c r="C81" s="30"/>
+      <c r="D81" s="30"/>
+      <c r="E81" s="30"/>
+      <c r="F81" s="30"/>
+      <c r="G81" s="30"/>
+      <c r="H81" s="30"/>
+      <c r="I81" s="30"/>
+      <c r="J81" s="30"/>
+      <c r="K81" s="30"/>
+      <c r="L81" s="30"/>
+      <c r="M81" s="30"/>
+      <c r="N81" s="30"/>
+      <c r="O81" s="30"/>
+      <c r="P81" s="30"/>
+      <c r="Q81" s="30"/>
+      <c r="R81" s="30"/>
+      <c r="S81" s="30"/>
     </row>
     <row r="82" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C82" s="31"/>
-      <c r="D82" s="31"/>
-      <c r="E82" s="31"/>
-      <c r="F82" s="31"/>
-      <c r="G82" s="31"/>
-      <c r="H82" s="31"/>
-      <c r="I82" s="31"/>
-      <c r="J82" s="31"/>
-      <c r="K82" s="31"/>
-      <c r="L82" s="31"/>
-      <c r="M82" s="31"/>
-      <c r="N82" s="31"/>
-      <c r="O82" s="31"/>
-      <c r="P82" s="31"/>
-      <c r="Q82" s="31"/>
-      <c r="R82" s="31"/>
-      <c r="S82" s="31"/>
+      <c r="C82" s="30"/>
+      <c r="D82" s="30"/>
+      <c r="E82" s="30"/>
+      <c r="F82" s="30"/>
+      <c r="G82" s="30"/>
+      <c r="H82" s="30"/>
+      <c r="I82" s="30"/>
+      <c r="J82" s="30"/>
+      <c r="K82" s="30"/>
+      <c r="L82" s="30"/>
+      <c r="M82" s="30"/>
+      <c r="N82" s="30"/>
+      <c r="O82" s="30"/>
+      <c r="P82" s="30"/>
+      <c r="Q82" s="30"/>
+      <c r="R82" s="30"/>
+      <c r="S82" s="30"/>
     </row>
     <row r="83" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C83" s="31"/>
-      <c r="D83" s="31"/>
-      <c r="E83" s="31"/>
-      <c r="F83" s="31"/>
-      <c r="G83" s="31"/>
-      <c r="H83" s="31"/>
-      <c r="I83" s="31"/>
-      <c r="J83" s="31"/>
-      <c r="K83" s="31"/>
-      <c r="L83" s="31"/>
-      <c r="M83" s="31"/>
-      <c r="N83" s="31"/>
-      <c r="O83" s="31"/>
-      <c r="P83" s="31"/>
-      <c r="Q83" s="31"/>
-      <c r="R83" s="31"/>
-      <c r="S83" s="31"/>
+      <c r="C83" s="30"/>
+      <c r="D83" s="30"/>
+      <c r="E83" s="30"/>
+      <c r="F83" s="30"/>
+      <c r="G83" s="30"/>
+      <c r="H83" s="30"/>
+      <c r="I83" s="30"/>
+      <c r="J83" s="30"/>
+      <c r="K83" s="30"/>
+      <c r="L83" s="30"/>
+      <c r="M83" s="30"/>
+      <c r="N83" s="30"/>
+      <c r="O83" s="30"/>
+      <c r="P83" s="30"/>
+      <c r="Q83" s="30"/>
+      <c r="R83" s="30"/>
+      <c r="S83" s="30"/>
     </row>
     <row r="84" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C84" s="31"/>
-      <c r="D84" s="31"/>
-      <c r="E84" s="31"/>
-      <c r="F84" s="31"/>
-      <c r="G84" s="31"/>
-      <c r="H84" s="31"/>
-      <c r="I84" s="31"/>
-      <c r="J84" s="31"/>
-      <c r="K84" s="31"/>
-      <c r="L84" s="31"/>
-      <c r="M84" s="31"/>
-      <c r="N84" s="31"/>
-      <c r="O84" s="31"/>
-      <c r="P84" s="31"/>
-      <c r="Q84" s="31"/>
-      <c r="R84" s="31"/>
-      <c r="S84" s="31"/>
+      <c r="C84" s="30"/>
+      <c r="D84" s="30"/>
+      <c r="E84" s="30"/>
+      <c r="F84" s="30"/>
+      <c r="G84" s="30"/>
+      <c r="H84" s="30"/>
+      <c r="I84" s="30"/>
+      <c r="J84" s="30"/>
+      <c r="K84" s="30"/>
+      <c r="L84" s="30"/>
+      <c r="M84" s="30"/>
+      <c r="N84" s="30"/>
+      <c r="O84" s="30"/>
+      <c r="P84" s="30"/>
+      <c r="Q84" s="30"/>
+      <c r="R84" s="30"/>
+      <c r="S84" s="30"/>
     </row>
     <row r="85" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C85" s="31"/>
-      <c r="D85" s="31"/>
-      <c r="E85" s="31"/>
-      <c r="F85" s="31"/>
-      <c r="G85" s="31"/>
-      <c r="H85" s="31"/>
-      <c r="I85" s="31"/>
-      <c r="J85" s="31"/>
-      <c r="K85" s="31"/>
-      <c r="L85" s="31"/>
-      <c r="M85" s="31"/>
-      <c r="N85" s="31"/>
-      <c r="O85" s="31"/>
-      <c r="P85" s="31"/>
-      <c r="Q85" s="31"/>
-      <c r="R85" s="31"/>
-      <c r="S85" s="31"/>
+      <c r="C85" s="30"/>
+      <c r="D85" s="30"/>
+      <c r="E85" s="30"/>
+      <c r="F85" s="30"/>
+      <c r="G85" s="30"/>
+      <c r="H85" s="30"/>
+      <c r="I85" s="30"/>
+      <c r="J85" s="30"/>
+      <c r="K85" s="30"/>
+      <c r="L85" s="30"/>
+      <c r="M85" s="30"/>
+      <c r="N85" s="30"/>
+      <c r="O85" s="30"/>
+      <c r="P85" s="30"/>
+      <c r="Q85" s="30"/>
+      <c r="R85" s="30"/>
+      <c r="S85" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2909,6 +2969,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>